<commit_message>
Indicadores: sumar la columna de enero-27 al REM
El REM publica el mes en curso y los seis siguientes; la planilla venía cortando
en seis, así que se perdía el último. Se agrega enero-27 en los tres bloques, con
los valores del relevamiento de julio-26: inflación 1,7%, TC 1.688, TAMAR 22,10%.

Los tres consumidores —senderoCER, senderoDL y senderoTAMAR— recorren los headers
y ruedan el año cuando el mes vuelve a enero, así que la columna nueva entra sin
tocar código. Justamente el caso del rollover es el que ejercita: hasta ahora
ninguna planilla lo había cruzado.

Para el BEI enero suma un forward más, y de los computables: cae dentro del tramo
donde hay bonos en las dos curvas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Indicadores.xlsx
+++ b/Indicadores.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="11">
   <si>
     <t>Julio</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>Diciembre</t>
+  </si>
+  <si>
+    <t>Enero</t>
   </si>
 </sst>
 </file>
@@ -447,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19417159-0C2D-4FF1-A703-3FC408462AE5}">
-  <dimension ref="A2:G12"/>
+  <dimension ref="A2:H12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -455,7 +458,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -475,10 +478,13 @@
         <v>9</v>
       </c>
       <c r="G3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -498,6 +504,9 @@
         <v>1.8</v>
       </c>
       <c r="G4" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="H4" s="1">
         <v>21.8</v>
       </c>
     </row>
@@ -506,7 +515,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -526,10 +535,13 @@
         <v>9</v>
       </c>
       <c r="G7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1470</v>
       </c>
@@ -549,6 +561,9 @@
         <v>1652</v>
       </c>
       <c r="G8">
+        <v>1688</v>
+      </c>
+      <c r="H8">
         <v>1859</v>
       </c>
     </row>
@@ -557,7 +572,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -577,10 +592,13 @@
         <v>9</v>
       </c>
       <c r="G11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>22.5</v>
       </c>
@@ -600,6 +618,9 @@
         <v>22.2</v>
       </c>
       <c r="G12" s="1">
+        <v>22.1</v>
+      </c>
+      <c r="H12" s="1">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Indicadores: sacar julio del REM, que ya no es pronóstico
El INDEC publicó el IPC de julio el 13-08-2026: 2,1% mensual, 33,8% interanual y
19,3% acumulado en el año. El REM de julio-26 lo proyectaba en 2,0%, así que se
pasó por 0,1 pp.

Con el dato publicado, julio deja de ser una fila de pronóstico y sale de los tres
bloques. Quedan agosto a enero más la de 12 meses.

Eso además limpia el aviso del BEI en Sendero CER, que aparecía justamente porque
había un mes ya cerrado en la planilla. El resto de las filas no se mueve: los
horizontes se anclan al calendario desde el nombre del mes, no a la posición de la
columna, así que correr todo una posición a la izquierda no cambia ningún cálculo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Indicadores.xlsx
+++ b/Indicadores.xlsx
@@ -1,101 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/franciscogranda/Desktop/Balanz/Monitores AI/Monitor Renta Fija ARG/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99417B1-AD27-924B-AA2E-2147A57C137C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="19420" windowHeight="10420" xr2:uid="{2A1DE20B-9174-463B-B235-59454B6DEAC4}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="19420" windowHeight="10420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Indicadores" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="11">
-  <si>
-    <t>Julio</t>
-  </si>
-  <si>
-    <t>Agosto</t>
-  </si>
-  <si>
-    <t>12 Meses</t>
-  </si>
-  <si>
-    <t>Octubre</t>
-  </si>
-  <si>
-    <t>Septiembre</t>
-  </si>
-  <si>
-    <t>REM inflación</t>
-  </si>
-  <si>
-    <t>REM tipo de cambio</t>
-  </si>
-  <si>
-    <t>Noviembre</t>
-  </si>
-  <si>
-    <t>REM tamar</t>
-  </si>
-  <si>
-    <t>Diciembre</t>
-  </si>
-  <si>
-    <t>Enero</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -114,22 +52,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -449,178 +446,197 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19417159-0C2D-4FF1-A703-3FC408462AE5}">
-  <dimension ref="A2:H12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>12 Meses</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" t="s">
-        <v>2</v>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>21.8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="D4" s="1">
-        <v>1.7</v>
-      </c>
-      <c r="E4" s="1">
-        <v>1.6</v>
-      </c>
-      <c r="F4" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="G4" s="1">
-        <v>1.7</v>
-      </c>
-      <c r="H4" s="1">
-        <v>21.8</v>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>12 Meses</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>6</v>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1512</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1546</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1577</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1618</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1652</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1688</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1859</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H7" t="s">
-        <v>2</v>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>12 Meses</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>1470</v>
-      </c>
-      <c r="B8">
-        <v>1512</v>
-      </c>
-      <c r="C8">
-        <v>1546</v>
-      </c>
-      <c r="D8">
-        <v>1577</v>
-      </c>
-      <c r="E8">
-        <v>1618</v>
-      </c>
-      <c r="F8">
-        <v>1652</v>
-      </c>
-      <c r="G8">
-        <v>1688</v>
-      </c>
-      <c r="H8">
-        <v>1859</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>22.5</v>
-      </c>
-      <c r="B12" s="1">
+    <row r="12">
+      <c r="A12" s="1" t="n">
         <v>22.4</v>
       </c>
-      <c r="C12" s="1">
+      <c r="B12" s="1" t="n">
         <v>22.72</v>
       </c>
-      <c r="D12" s="1">
+      <c r="C12" s="1" t="n">
         <v>22.3</v>
       </c>
-      <c r="E12" s="1">
+      <c r="D12" s="1" t="n">
         <v>22.1</v>
       </c>
-      <c r="F12" s="1">
+      <c r="E12" s="1" t="n">
         <v>22.2</v>
       </c>
-      <c r="G12" s="1">
+      <c r="F12" s="1" t="n">
         <v>22.1</v>
       </c>
-      <c r="H12" s="1">
+      <c r="G12" s="1" t="n">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Indicadores: arreglar el borrado de julio, que se había llevado las etiquetas
El commit anterior usó delete_cols(1) para sacar la columna de julio, pero las
etiquetas de bloque —'REM inflación', 'REM tipo de cambio', 'REM tamar'— viven en
A2, A6 y A10, o sea en esa misma columna. Se fueron con ella y los tres parsers
dejaron de encontrar los bloques: la tabla del BEI quedaba vacía.

Ahora se corren una posición a la izquierda SÓLO las filas de headers y de
valores, y las etiquetas quedan donde estaban.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Indicadores.xlsx
+++ b/Indicadores.xlsx
@@ -451,11 +451,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A2:H12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REM inflación</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -515,9 +520,15 @@
       <c r="G4" s="1" t="n">
         <v>21.8</v>
       </c>
-    </row>
-    <row r="5"/>
-    <row r="6"/>
+      <c r="H4" s="1" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REM tipo de cambio</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -578,8 +589,13 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>REM tamar</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -639,6 +655,7 @@
       <c r="G12" s="1" t="n">
         <v>22</v>
       </c>
+      <c r="H12" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
REM: la ventana de inflación pasa a septiembre-febrero
El BCRA publicó el CER hasta el 15/10, que es el período que ajusta con el IPC de agosto (1,7%;
del 15/09 al 15/10 el CER sube exactamente 1,700%). Agosto ya no hace falta en la fila: la fila
de inflación del REM de agosto-26 queda de septiembre a febrero, alineada con el «12 Meses»
(variación interanual a ago-27). Tipo de cambio y TAMAR ya arrancaban en septiembre.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Indicadores.xlsx
+++ b/Indicadores.xlsx
@@ -464,32 +464,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Septiembre</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Septiembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Diciembre</t>
+          <t>Enero</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Enero</t>
+          <t>Febrero</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -500,19 +500,19 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="B4" s="1" t="n">
         <v>1.7</v>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>1.8</v>
-      </c>
       <c r="C4" s="1" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="D4" s="1" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="E4" s="1" t="n">
         <v>1.6</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>1.78</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>1.6</v>

</xml_diff>